<commit_message>
feat: actualizar plantilla de excel de recepcion
</commit_message>
<xml_diff>
--- a/pesaje/analytica/Report/Recepcion-Export-Pesaje-Base.xlsx
+++ b/pesaje/analytica/Report/Recepcion-Export-Pesaje-Base.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-project-configuration\pesaje\analytica\Report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-pesaje-api\Acopio.Pesaje.Apis\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A39CC78-CD3B-4534-A3AB-F5CDC7010739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10205B83-766B-4C65-A6D4-416991B76EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Analytica Mineral Services Sac</t>
   </si>
@@ -39,12 +39,27 @@
     <t>Exportado por:</t>
   </si>
   <si>
+    <t>FECHA PESADO</t>
+  </si>
+  <si>
+    <t>PROVEEDOR</t>
+  </si>
+  <si>
+    <t>SUCURSAL</t>
+  </si>
+  <si>
     <t>,</t>
   </si>
   <si>
+    <t>RUC</t>
+  </si>
+  <si>
     <t>FECHA INGRESO</t>
   </si>
   <si>
+    <t>NRO TICKET</t>
+  </si>
+  <si>
     <t>TRANSPORTISTA</t>
   </si>
   <si>
@@ -63,13 +78,28 @@
     <t>PESO NETO</t>
   </si>
   <si>
+    <t>PESAJE LIBRE</t>
+  </si>
+  <si>
+    <t>MOTIVO</t>
+  </si>
+  <si>
+    <t>ESTADO PESAJE LIBRE</t>
+  </si>
+  <si>
+    <t>PLACA</t>
+  </si>
+  <si>
     <t>PRODUCTO</t>
   </si>
   <si>
+    <t>GUARDIA</t>
+  </si>
+  <si>
+    <t>TURNO</t>
+  </si>
+  <si>
     <t>ENVASE</t>
-  </si>
-  <si>
-    <t>PLACA</t>
   </si>
 </sst>
 </file>
@@ -80,7 +110,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-&quot;S/ &quot;* #,##0.00_-;&quot;-S/ &quot;* #,##0.00_-;_-&quot;S/ &quot;* \-??_-;_-@_-"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -543,23 +573,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AO11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4"/>
+  <dimension ref="A1:AR11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.6640625" style="4" customWidth="1"/>
     <col min="2" max="2" width="19.5546875" style="4" customWidth="1"/>
     <col min="3" max="3" width="52.21875" style="4" customWidth="1"/>
     <col min="4" max="4" width="17.33203125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="23.88671875" style="4" customWidth="1"/>
-    <col min="6" max="6" width="28.44140625" style="4" customWidth="1"/>
-    <col min="7" max="7" width="25.77734375" style="4" customWidth="1"/>
-    <col min="8" max="8" width="28.5546875" style="4" customWidth="1"/>
-    <col min="9" max="9" width="24.77734375" style="4" customWidth="1"/>
-    <col min="10" max="11" width="14.88671875" style="4" customWidth="1"/>
-    <col min="12" max="19" width="24.6640625" style="4" customWidth="1"/>
+    <col min="5" max="7" width="23.88671875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="28.44140625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="25.77734375" style="4" customWidth="1"/>
+    <col min="10" max="10" width="28.5546875" style="4" customWidth="1"/>
+    <col min="11" max="11" width="24.77734375" style="4" customWidth="1"/>
+    <col min="12" max="12" width="45.5546875" style="4" customWidth="1"/>
+    <col min="13" max="13" width="43.6640625" style="4" customWidth="1"/>
+    <col min="14" max="22" width="24.6640625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41">
+    <row r="1" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A1" s="5"/>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -579,9 +610,9 @@
       <c r="Q1" s="5"/>
       <c r="R1" s="5"/>
       <c r="S1" s="5"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
@@ -601,8 +632,11 @@
       <c r="AM1" s="1"/>
       <c r="AN1" s="1"/>
       <c r="AO1" s="1"/>
+      <c r="AP1" s="1"/>
+      <c r="AQ1" s="1"/>
+      <c r="AR1" s="1"/>
     </row>
-    <row r="2" spans="1:41" ht="48.75" customHeight="1">
+    <row r="2" spans="1:44" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
@@ -614,19 +648,19 @@
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
       <c r="I2" s="13"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
       <c r="L2" s="6"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
       <c r="O2" s="5"/>
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
       <c r="R2" s="5"/>
       <c r="S2" s="5"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
+      <c r="T2" s="5"/>
+      <c r="U2" s="5"/>
+      <c r="V2" s="5"/>
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
@@ -646,8 +680,11 @@
       <c r="AM2" s="1"/>
       <c r="AN2" s="1"/>
       <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
     </row>
-    <row r="3" spans="1:41" ht="22.5" customHeight="1">
+    <row r="3" spans="1:44" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>1</v>
       </c>
@@ -659,19 +696,19 @@
       <c r="G3" s="14"/>
       <c r="H3" s="14"/>
       <c r="I3" s="14"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
       <c r="L3" s="7"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
       <c r="S3" s="5"/>
-      <c r="T3" s="1"/>
-      <c r="U3" s="1"/>
-      <c r="V3" s="1"/>
+      <c r="T3" s="5"/>
+      <c r="U3" s="5"/>
+      <c r="V3" s="5"/>
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
@@ -691,8 +728,11 @@
       <c r="AM3" s="1"/>
       <c r="AN3" s="1"/>
       <c r="AO3" s="1"/>
+      <c r="AP3" s="1"/>
+      <c r="AQ3" s="1"/>
+      <c r="AR3" s="1"/>
     </row>
-    <row r="4" spans="1:41" ht="15.75" customHeight="1">
+    <row r="4" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -704,17 +744,17 @@
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
       <c r="Q4" s="5"/>
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
-      <c r="T4" s="1"/>
-      <c r="U4" s="1"/>
-      <c r="V4" s="1"/>
+      <c r="T4" s="5"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="5"/>
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
@@ -734,8 +774,11 @@
       <c r="AM4" s="1"/>
       <c r="AN4" s="1"/>
       <c r="AO4" s="1"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="1"/>
+      <c r="AR4" s="1"/>
     </row>
-    <row r="5" spans="1:41" ht="18">
+    <row r="5" spans="1:44" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -747,9 +790,11 @@
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
-      <c r="L5" s="9"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="9"/>
     </row>
-    <row r="6" spans="1:41" ht="18">
+    <row r="6" spans="1:44" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="9"/>
       <c r="B6" s="10" t="s">
         <v>2</v>
@@ -761,9 +806,10 @@
       <c r="G6" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="L6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="N6" s="9"/>
     </row>
-    <row r="7" spans="1:41" ht="18">
+    <row r="7" spans="1:44" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -776,73 +822,84 @@
       <c r="J7" s="9"/>
       <c r="K7" s="9"/>
       <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
     </row>
-    <row r="8" spans="1:41" s="11" customFormat="1">
+    <row r="8" spans="1:44" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="U8" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:44" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="H11" s="4" t="s">
         <v>7</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="O8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="P8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="R8" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:41" s="4" customFormat="1"/>
-    <row r="11" spans="1:41">
-      <c r="F11" s="4" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>